<commit_message>
Literature review pots-review check
</commit_message>
<xml_diff>
--- a/Data/0_Review/Literature_review.xlsx
+++ b/Data/0_Review/Literature_review.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/auger-methe/Sync/GitHub/InformedHSA/Data/0_Review/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEFF4045-1F12-F548-B09A-CAC3C6F28328}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8395ECA-CA2C-354D-AE9D-41FFFAE22153}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3200" yWindow="500" windowWidth="48000" windowHeight="9180" xr2:uid="{C9BFA348-15B8-4AE0-B546-034C584F196E}"/>
+    <workbookView xWindow="3200" yWindow="500" windowWidth="48000" windowHeight="19320" xr2:uid="{C9BFA348-15B8-4AE0-B546-034C584F196E}"/>
   </bookViews>
   <sheets>
     <sheet name="Documents" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3053" uniqueCount="1343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3067" uniqueCount="1346">
   <si>
     <t>Authors</t>
   </si>
@@ -4719,6 +4719,15 @@
   </si>
   <si>
     <t>Does the habitat selection analysis account for individual (e.g., via random effect or separate analyses)?</t>
+  </si>
+  <si>
+    <t>Kodiak brown bear</t>
+  </si>
+  <si>
+    <t>Ursus Arctos</t>
+  </si>
+  <si>
+    <t>"Our modeling efforts highlight the importance of behavior-specific resource selection and connectivity across the landscape. Collectively, the results of this analysis accurately identified factors influencing bear travel during the salmon stream spawning season and provide managers with information to make informed decisions to conserve bear connectivity. Our results demonstrated that during a critical period of foraging, the stream spawning season, bears used relatively few paths to travel among foraging sites and these corridors were often centered near lake edges and areas with narrow topographic relief that facilitated movement. Maintaining the integrity of these travel corridors is critical to the conservation and management of the Kodiak brown bear. To achieve the management goals of maintaining a high population level and body size of Kodiak brown bears, ADF&amp;G and the Kodiak NWR must take steps to ensure that travel corridors are maintained by identifying travel routes and ensuring the future integrity of those routes."</t>
   </si>
 </sst>
 </file>
@@ -4853,7 +4862,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -4884,6 +4893,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5198,7 +5210,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{965273D1-CF78-4D09-8A99-E1B085961B00}">
-  <dimension ref="A1:W334"/>
+  <dimension ref="A1:X333"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
@@ -9761,7 +9773,7 @@
         <v>1286</v>
       </c>
     </row>
-    <row r="65" spans="1:23">
+    <row r="65" spans="1:24">
       <c r="A65" t="s">
         <v>460</v>
       </c>
@@ -9832,7 +9844,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="66" spans="1:23">
+    <row r="66" spans="1:24">
       <c r="A66" t="s">
         <v>475</v>
       </c>
@@ -9903,7 +9915,7 @@
         <v>1293</v>
       </c>
     </row>
-    <row r="67" spans="1:23">
+    <row r="67" spans="1:24">
       <c r="A67" t="s">
         <v>482</v>
       </c>
@@ -9974,7 +9986,7 @@
         <v>1298</v>
       </c>
     </row>
-    <row r="68" spans="1:23">
+    <row r="68" spans="1:24">
       <c r="A68" t="s">
         <v>485</v>
       </c>
@@ -10045,7 +10057,7 @@
         <v>1299</v>
       </c>
     </row>
-    <row r="69" spans="1:23">
+    <row r="69" spans="1:24">
       <c r="A69" t="s">
         <v>488</v>
       </c>
@@ -10116,7 +10128,7 @@
         <v>1302</v>
       </c>
     </row>
-    <row r="70" spans="1:23" ht="16">
+    <row r="70" spans="1:24" ht="16">
       <c r="A70" t="s">
         <v>492</v>
       </c>
@@ -10187,7 +10199,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="71" spans="1:23">
+    <row r="71" spans="1:24">
       <c r="A71" t="s">
         <v>498</v>
       </c>
@@ -10258,7 +10270,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="72" spans="1:23" ht="16">
+    <row r="72" spans="1:24" ht="16">
       <c r="A72" s="16" t="s">
         <v>506</v>
       </c>
@@ -10329,7 +10341,79 @@
         <v>66</v>
       </c>
     </row>
-    <row r="80" spans="1:23" ht="18">
+    <row r="73" spans="1:24" s="24" customFormat="1">
+      <c r="A73" s="24" t="s">
+        <v>562</v>
+      </c>
+      <c r="B73" s="24" t="s">
+        <v>1037</v>
+      </c>
+      <c r="C73" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="D73" s="24">
+        <v>12</v>
+      </c>
+      <c r="E73" s="24">
+        <v>1</v>
+      </c>
+      <c r="F73" s="24">
+        <v>2024</v>
+      </c>
+      <c r="G73" s="24" t="s">
+        <v>564</v>
+      </c>
+      <c r="H73" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="I73" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="J73" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="K73" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="L73" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="M73" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="N73" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="O73" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="P73" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q73" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="R73" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="S73" s="26" t="s">
+        <v>40</v>
+      </c>
+      <c r="T73" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="U73" s="26" t="s">
+        <v>1345</v>
+      </c>
+      <c r="V73" s="26" t="s">
+        <v>1343</v>
+      </c>
+      <c r="W73" s="26" t="s">
+        <v>1344</v>
+      </c>
+      <c r="X73" s="26"/>
+    </row>
+    <row r="80" spans="1:24" ht="18">
       <c r="A80" s="5" t="s">
         <v>511</v>
       </c>
@@ -15872,25 +15956,25 @@
     </row>
     <row r="259" spans="1:9">
       <c r="A259" t="s">
-        <v>562</v>
+        <v>1038</v>
       </c>
       <c r="B259" t="s">
-        <v>1037</v>
+        <v>1039</v>
       </c>
       <c r="C259" t="s">
-        <v>93</v>
+        <v>1040</v>
       </c>
       <c r="D259">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E259">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F259">
         <v>2024</v>
       </c>
       <c r="G259" t="s">
-        <v>564</v>
+        <v>1041</v>
       </c>
       <c r="H259" s="1" t="s">
         <v>23</v>
@@ -15901,25 +15985,25 @@
     </row>
     <row r="260" spans="1:9">
       <c r="A260" t="s">
-        <v>1038</v>
+        <v>1042</v>
       </c>
       <c r="B260" t="s">
-        <v>1039</v>
+        <v>1043</v>
       </c>
       <c r="C260" t="s">
-        <v>1040</v>
-      </c>
-      <c r="D260">
-        <v>15</v>
-      </c>
-      <c r="E260">
-        <v>4</v>
+        <v>1044</v>
+      </c>
+      <c r="D260" t="s">
+        <v>47</v>
+      </c>
+      <c r="E260" t="s">
+        <v>47</v>
       </c>
       <c r="F260">
         <v>2024</v>
       </c>
       <c r="G260" t="s">
-        <v>1041</v>
+        <v>1045</v>
       </c>
       <c r="H260" s="1" t="s">
         <v>23</v>
@@ -15930,25 +16014,25 @@
     </row>
     <row r="261" spans="1:9">
       <c r="A261" t="s">
-        <v>1042</v>
+        <v>1046</v>
       </c>
       <c r="B261" t="s">
-        <v>1043</v>
+        <v>1047</v>
       </c>
       <c r="C261" t="s">
-        <v>1044</v>
-      </c>
-      <c r="D261" t="s">
-        <v>47</v>
-      </c>
-      <c r="E261" t="s">
-        <v>47</v>
+        <v>327</v>
+      </c>
+      <c r="D261">
+        <v>5</v>
+      </c>
+      <c r="E261">
+        <v>4</v>
       </c>
       <c r="F261">
         <v>2024</v>
       </c>
       <c r="G261" t="s">
-        <v>1045</v>
+        <v>1048</v>
       </c>
       <c r="H261" s="1" t="s">
         <v>23</v>
@@ -15959,25 +16043,25 @@
     </row>
     <row r="262" spans="1:9">
       <c r="A262" t="s">
-        <v>1046</v>
+        <v>1049</v>
       </c>
       <c r="B262" t="s">
-        <v>1047</v>
+        <v>1050</v>
       </c>
       <c r="C262" t="s">
-        <v>327</v>
+        <v>1051</v>
       </c>
       <c r="D262">
-        <v>5</v>
-      </c>
-      <c r="E262">
-        <v>4</v>
+        <v>219</v>
+      </c>
+      <c r="E262" t="s">
+        <v>47</v>
       </c>
       <c r="F262">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="G262" t="s">
-        <v>1048</v>
+        <v>1052</v>
       </c>
       <c r="H262" s="1" t="s">
         <v>23</v>
@@ -15988,25 +16072,25 @@
     </row>
     <row r="263" spans="1:9">
       <c r="A263" t="s">
-        <v>1049</v>
+        <v>1053</v>
       </c>
       <c r="B263" t="s">
-        <v>1050</v>
+        <v>1054</v>
       </c>
       <c r="C263" t="s">
-        <v>1051</v>
+        <v>1055</v>
       </c>
       <c r="D263">
-        <v>219</v>
+        <v>80</v>
       </c>
       <c r="E263" t="s">
         <v>47</v>
       </c>
       <c r="F263">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="G263" t="s">
-        <v>1052</v>
+        <v>1056</v>
       </c>
       <c r="H263" s="1" t="s">
         <v>23</v>
@@ -16017,25 +16101,25 @@
     </row>
     <row r="264" spans="1:9">
       <c r="A264" t="s">
-        <v>1053</v>
+        <v>592</v>
       </c>
       <c r="B264" t="s">
-        <v>1054</v>
+        <v>593</v>
       </c>
       <c r="C264" t="s">
-        <v>1055</v>
+        <v>1057</v>
       </c>
       <c r="D264">
-        <v>80</v>
-      </c>
-      <c r="E264" t="s">
-        <v>47</v>
+        <v>71</v>
+      </c>
+      <c r="E264">
+        <v>1</v>
       </c>
       <c r="F264">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="G264" t="s">
-        <v>1056</v>
+        <v>594</v>
       </c>
       <c r="H264" s="1" t="s">
         <v>23</v>
@@ -16046,25 +16130,25 @@
     </row>
     <row r="265" spans="1:9">
       <c r="A265" t="s">
-        <v>592</v>
+        <v>1058</v>
       </c>
       <c r="B265" t="s">
-        <v>593</v>
+        <v>1059</v>
       </c>
       <c r="C265" t="s">
-        <v>1057</v>
+        <v>1060</v>
       </c>
       <c r="D265">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="E265">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F265">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="G265" t="s">
-        <v>594</v>
+        <v>1061</v>
       </c>
       <c r="H265" s="1" t="s">
         <v>23</v>
@@ -16075,25 +16159,25 @@
     </row>
     <row r="266" spans="1:9">
       <c r="A266" t="s">
-        <v>1058</v>
+        <v>615</v>
       </c>
       <c r="B266" t="s">
-        <v>1059</v>
+        <v>1062</v>
       </c>
       <c r="C266" t="s">
-        <v>1060</v>
+        <v>617</v>
       </c>
       <c r="D266">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="E266">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F266">
         <v>2024</v>
       </c>
       <c r="G266" t="s">
-        <v>1061</v>
+        <v>618</v>
       </c>
       <c r="H266" s="1" t="s">
         <v>23</v>
@@ -16104,25 +16188,25 @@
     </row>
     <row r="267" spans="1:9">
       <c r="A267" t="s">
-        <v>615</v>
+        <v>1063</v>
       </c>
       <c r="B267" t="s">
-        <v>1062</v>
+        <v>1064</v>
       </c>
       <c r="C267" t="s">
-        <v>617</v>
+        <v>230</v>
       </c>
       <c r="D267">
-        <v>44</v>
-      </c>
-      <c r="E267">
-        <v>6</v>
+        <v>299</v>
+      </c>
+      <c r="E267" t="s">
+        <v>47</v>
       </c>
       <c r="F267">
         <v>2024</v>
       </c>
       <c r="G267" t="s">
-        <v>618</v>
+        <v>1065</v>
       </c>
       <c r="H267" s="1" t="s">
         <v>23</v>
@@ -16133,25 +16217,25 @@
     </row>
     <row r="268" spans="1:9">
       <c r="A268" t="s">
-        <v>1063</v>
+        <v>1066</v>
       </c>
       <c r="B268" t="s">
-        <v>1064</v>
+        <v>1067</v>
       </c>
       <c r="C268" t="s">
-        <v>230</v>
+        <v>1068</v>
       </c>
       <c r="D268">
-        <v>299</v>
-      </c>
-      <c r="E268" t="s">
-        <v>47</v>
+        <v>25</v>
+      </c>
+      <c r="E268">
+        <v>6</v>
       </c>
       <c r="F268">
         <v>2024</v>
       </c>
       <c r="G268" t="s">
-        <v>1065</v>
+        <v>1069</v>
       </c>
       <c r="H268" s="1" t="s">
         <v>23</v>
@@ -16162,25 +16246,25 @@
     </row>
     <row r="269" spans="1:9">
       <c r="A269" t="s">
-        <v>1066</v>
+        <v>1070</v>
       </c>
       <c r="B269" t="s">
-        <v>1067</v>
+        <v>1071</v>
       </c>
       <c r="C269" t="s">
-        <v>1068</v>
-      </c>
-      <c r="D269">
-        <v>25</v>
-      </c>
-      <c r="E269">
-        <v>6</v>
+        <v>1072</v>
+      </c>
+      <c r="D269" t="s">
+        <v>47</v>
+      </c>
+      <c r="E269" t="s">
+        <v>47</v>
       </c>
       <c r="F269">
         <v>2024</v>
       </c>
       <c r="G269" t="s">
-        <v>1069</v>
+        <v>1073</v>
       </c>
       <c r="H269" s="1" t="s">
         <v>23</v>
@@ -16191,25 +16275,25 @@
     </row>
     <row r="270" spans="1:9">
       <c r="A270" t="s">
-        <v>1070</v>
+        <v>1074</v>
       </c>
       <c r="B270" t="s">
-        <v>1071</v>
+        <v>1075</v>
       </c>
       <c r="C270" t="s">
-        <v>1072</v>
-      </c>
-      <c r="D270" t="s">
-        <v>47</v>
-      </c>
-      <c r="E270" t="s">
-        <v>47</v>
+        <v>477</v>
+      </c>
+      <c r="D270">
+        <v>93</v>
+      </c>
+      <c r="E270">
+        <v>7</v>
       </c>
       <c r="F270">
         <v>2024</v>
       </c>
       <c r="G270" t="s">
-        <v>1073</v>
+        <v>1076</v>
       </c>
       <c r="H270" s="1" t="s">
         <v>23</v>
@@ -16220,25 +16304,25 @@
     </row>
     <row r="271" spans="1:9">
       <c r="A271" t="s">
-        <v>1074</v>
+        <v>1077</v>
       </c>
       <c r="B271" t="s">
-        <v>1075</v>
+        <v>1078</v>
       </c>
       <c r="C271" t="s">
-        <v>477</v>
+        <v>744</v>
       </c>
       <c r="D271">
-        <v>93</v>
+        <v>16</v>
       </c>
       <c r="E271">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="F271">
         <v>2024</v>
       </c>
       <c r="G271" t="s">
-        <v>1076</v>
+        <v>1079</v>
       </c>
       <c r="H271" s="1" t="s">
         <v>23</v>
@@ -16249,25 +16333,25 @@
     </row>
     <row r="272" spans="1:9">
       <c r="A272" t="s">
-        <v>1077</v>
+        <v>1080</v>
       </c>
       <c r="B272" t="s">
-        <v>1078</v>
+        <v>1081</v>
       </c>
       <c r="C272" t="s">
-        <v>744</v>
+        <v>1082</v>
       </c>
       <c r="D272">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="E272">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="F272">
         <v>2024</v>
       </c>
       <c r="G272" t="s">
-        <v>1079</v>
+        <v>1083</v>
       </c>
       <c r="H272" s="1" t="s">
         <v>23</v>
@@ -16278,25 +16362,25 @@
     </row>
     <row r="273" spans="1:9">
       <c r="A273" t="s">
-        <v>1080</v>
+        <v>1084</v>
       </c>
       <c r="B273" t="s">
-        <v>1081</v>
+        <v>1085</v>
       </c>
       <c r="C273" t="s">
-        <v>1082</v>
+        <v>1086</v>
       </c>
       <c r="D273">
-        <v>50</v>
-      </c>
-      <c r="E273">
-        <v>6</v>
+        <v>204</v>
+      </c>
+      <c r="E273" t="s">
+        <v>47</v>
       </c>
       <c r="F273">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="G273" t="s">
-        <v>1083</v>
+        <v>1087</v>
       </c>
       <c r="H273" s="1" t="s">
         <v>23</v>
@@ -16307,25 +16391,25 @@
     </row>
     <row r="274" spans="1:9">
       <c r="A274" t="s">
-        <v>1084</v>
+        <v>1088</v>
       </c>
       <c r="B274" t="s">
-        <v>1085</v>
+        <v>1089</v>
       </c>
       <c r="C274" t="s">
-        <v>1086</v>
+        <v>133</v>
       </c>
       <c r="D274">
-        <v>204</v>
-      </c>
-      <c r="E274" t="s">
-        <v>47</v>
+        <v>14</v>
+      </c>
+      <c r="E274">
+        <v>1</v>
       </c>
       <c r="F274">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="G274" t="s">
-        <v>1087</v>
+        <v>1090</v>
       </c>
       <c r="H274" s="1" t="s">
         <v>23</v>
@@ -16336,25 +16420,25 @@
     </row>
     <row r="275" spans="1:9">
       <c r="A275" t="s">
-        <v>1088</v>
+        <v>1091</v>
       </c>
       <c r="B275" t="s">
-        <v>1089</v>
+        <v>1092</v>
       </c>
       <c r="C275" t="s">
-        <v>133</v>
+        <v>740</v>
       </c>
       <c r="D275">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="E275">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F275">
         <v>2024</v>
       </c>
       <c r="G275" t="s">
-        <v>1090</v>
+        <v>1093</v>
       </c>
       <c r="H275" s="1" t="s">
         <v>23</v>
@@ -16365,25 +16449,25 @@
     </row>
     <row r="276" spans="1:9">
       <c r="A276" t="s">
-        <v>1091</v>
+        <v>1094</v>
       </c>
       <c r="B276" t="s">
-        <v>1092</v>
+        <v>1095</v>
       </c>
       <c r="C276" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="D276">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="E276">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F276">
         <v>2024</v>
       </c>
       <c r="G276" t="s">
-        <v>1093</v>
+        <v>1096</v>
       </c>
       <c r="H276" s="1" t="s">
         <v>23</v>
@@ -16394,25 +16478,25 @@
     </row>
     <row r="277" spans="1:9">
       <c r="A277" t="s">
-        <v>1094</v>
+        <v>1097</v>
       </c>
       <c r="B277" t="s">
-        <v>1095</v>
+        <v>1098</v>
       </c>
       <c r="C277" t="s">
-        <v>744</v>
+        <v>429</v>
       </c>
       <c r="D277">
-        <v>16</v>
-      </c>
-      <c r="E277">
-        <v>24</v>
+        <v>51</v>
+      </c>
+      <c r="E277" t="s">
+        <v>47</v>
       </c>
       <c r="F277">
         <v>2024</v>
       </c>
       <c r="G277" t="s">
-        <v>1096</v>
+        <v>1099</v>
       </c>
       <c r="H277" s="1" t="s">
         <v>23</v>
@@ -16423,25 +16507,25 @@
     </row>
     <row r="278" spans="1:9">
       <c r="A278" t="s">
-        <v>1097</v>
+        <v>1100</v>
       </c>
       <c r="B278" t="s">
-        <v>1098</v>
+        <v>1101</v>
       </c>
       <c r="C278" t="s">
-        <v>429</v>
+        <v>1102</v>
       </c>
       <c r="D278">
-        <v>51</v>
+        <v>282</v>
       </c>
       <c r="E278" t="s">
         <v>47</v>
       </c>
       <c r="F278">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="G278" t="s">
-        <v>1099</v>
+        <v>1103</v>
       </c>
       <c r="H278" s="1" t="s">
         <v>23</v>
@@ -16452,25 +16536,25 @@
     </row>
     <row r="279" spans="1:9">
       <c r="A279" t="s">
-        <v>1100</v>
+        <v>1104</v>
       </c>
       <c r="B279" t="s">
-        <v>1101</v>
+        <v>1105</v>
       </c>
       <c r="C279" t="s">
-        <v>1102</v>
+        <v>477</v>
       </c>
       <c r="D279">
-        <v>282</v>
-      </c>
-      <c r="E279" t="s">
-        <v>47</v>
+        <v>94</v>
+      </c>
+      <c r="E279">
+        <v>1</v>
       </c>
       <c r="F279">
         <v>2025</v>
       </c>
       <c r="G279" t="s">
-        <v>1103</v>
+        <v>1106</v>
       </c>
       <c r="H279" s="1" t="s">
         <v>23</v>
@@ -16481,25 +16565,25 @@
     </row>
     <row r="280" spans="1:9">
       <c r="A280" t="s">
-        <v>1104</v>
+        <v>1107</v>
       </c>
       <c r="B280" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="C280" t="s">
-        <v>477</v>
+        <v>1109</v>
       </c>
       <c r="D280">
-        <v>94</v>
+        <v>167</v>
       </c>
       <c r="E280">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F280">
         <v>2025</v>
       </c>
       <c r="G280" t="s">
-        <v>1106</v>
+        <v>1110</v>
       </c>
       <c r="H280" s="1" t="s">
         <v>23</v>
@@ -16510,25 +16594,25 @@
     </row>
     <row r="281" spans="1:9">
       <c r="A281" t="s">
-        <v>1107</v>
+        <v>1111</v>
       </c>
       <c r="B281" t="s">
-        <v>1108</v>
+        <v>1112</v>
       </c>
       <c r="C281" t="s">
-        <v>1109</v>
+        <v>1113</v>
       </c>
       <c r="D281">
-        <v>167</v>
+        <v>30</v>
       </c>
       <c r="E281">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F281">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="G281" t="s">
-        <v>1110</v>
+        <v>1114</v>
       </c>
       <c r="H281" s="1" t="s">
         <v>23</v>
@@ -16539,25 +16623,25 @@
     </row>
     <row r="282" spans="1:9">
       <c r="A282" t="s">
-        <v>1111</v>
+        <v>1115</v>
       </c>
       <c r="B282" t="s">
-        <v>1112</v>
+        <v>1116</v>
       </c>
       <c r="C282" t="s">
-        <v>1113</v>
+        <v>140</v>
       </c>
       <c r="D282">
-        <v>30</v>
+        <v>62</v>
       </c>
       <c r="E282">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F282">
-        <v>2024</v>
-      </c>
-      <c r="G282" t="s">
-        <v>1114</v>
+        <v>2025</v>
+      </c>
+      <c r="G282" s="7" t="s">
+        <v>1117</v>
       </c>
       <c r="H282" s="1" t="s">
         <v>23</v>
@@ -16568,25 +16652,25 @@
     </row>
     <row r="283" spans="1:9">
       <c r="A283" t="s">
-        <v>1115</v>
+        <v>1118</v>
       </c>
       <c r="B283" t="s">
-        <v>1116</v>
+        <v>1119</v>
       </c>
       <c r="C283" t="s">
-        <v>140</v>
+        <v>1120</v>
       </c>
       <c r="D283">
-        <v>62</v>
-      </c>
-      <c r="E283">
-        <v>4</v>
+        <v>262</v>
+      </c>
+      <c r="E283" t="s">
+        <v>47</v>
       </c>
       <c r="F283">
-        <v>2025</v>
-      </c>
-      <c r="G283" s="7" t="s">
-        <v>1117</v>
+        <v>2024</v>
+      </c>
+      <c r="G283" t="s">
+        <v>1121</v>
       </c>
       <c r="H283" s="1" t="s">
         <v>23</v>
@@ -16597,16 +16681,16 @@
     </row>
     <row r="284" spans="1:9">
       <c r="A284" t="s">
-        <v>1118</v>
+        <v>1122</v>
       </c>
       <c r="B284" t="s">
-        <v>1119</v>
+        <v>1123</v>
       </c>
       <c r="C284" t="s">
-        <v>1120</v>
+        <v>253</v>
       </c>
       <c r="D284">
-        <v>262</v>
+        <v>954</v>
       </c>
       <c r="E284" t="s">
         <v>47</v>
@@ -16615,7 +16699,7 @@
         <v>2024</v>
       </c>
       <c r="G284" t="s">
-        <v>1121</v>
+        <v>1124</v>
       </c>
       <c r="H284" s="1" t="s">
         <v>23</v>
@@ -16626,25 +16710,25 @@
     </row>
     <row r="285" spans="1:9">
       <c r="A285" t="s">
-        <v>1122</v>
+        <v>1125</v>
       </c>
       <c r="B285" t="s">
-        <v>1123</v>
+        <v>1126</v>
       </c>
       <c r="C285" t="s">
-        <v>253</v>
+        <v>35</v>
       </c>
       <c r="D285">
-        <v>954</v>
-      </c>
-      <c r="E285" t="s">
-        <v>47</v>
+        <v>14</v>
+      </c>
+      <c r="E285">
+        <v>8</v>
       </c>
       <c r="F285">
         <v>2024</v>
       </c>
       <c r="G285" t="s">
-        <v>1124</v>
+        <v>1127</v>
       </c>
       <c r="H285" s="1" t="s">
         <v>23</v>
@@ -16655,25 +16739,25 @@
     </row>
     <row r="286" spans="1:9">
       <c r="A286" t="s">
-        <v>1125</v>
+        <v>1128</v>
       </c>
       <c r="B286" t="s">
-        <v>1126</v>
+        <v>1129</v>
       </c>
       <c r="C286" t="s">
-        <v>35</v>
+        <v>93</v>
       </c>
       <c r="D286">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E286">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F286">
         <v>2024</v>
       </c>
       <c r="G286" t="s">
-        <v>1127</v>
+        <v>1130</v>
       </c>
       <c r="H286" s="1" t="s">
         <v>23</v>
@@ -16684,25 +16768,25 @@
     </row>
     <row r="287" spans="1:9">
       <c r="A287" t="s">
-        <v>1128</v>
+        <v>1131</v>
       </c>
       <c r="B287" t="s">
-        <v>1129</v>
+        <v>1132</v>
       </c>
       <c r="C287" t="s">
-        <v>93</v>
+        <v>1133</v>
       </c>
       <c r="D287">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E287">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F287">
         <v>2024</v>
       </c>
       <c r="G287" t="s">
-        <v>1130</v>
+        <v>1134</v>
       </c>
       <c r="H287" s="1" t="s">
         <v>23</v>
@@ -16713,25 +16797,25 @@
     </row>
     <row r="288" spans="1:9">
       <c r="A288" t="s">
-        <v>1131</v>
+        <v>1135</v>
       </c>
       <c r="B288" t="s">
-        <v>1132</v>
+        <v>1136</v>
       </c>
       <c r="C288" t="s">
-        <v>1133</v>
-      </c>
-      <c r="D288">
-        <v>13</v>
-      </c>
-      <c r="E288">
-        <v>8</v>
+        <v>1137</v>
+      </c>
+      <c r="D288" t="s">
+        <v>47</v>
+      </c>
+      <c r="E288" t="s">
+        <v>47</v>
       </c>
       <c r="F288">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="G288" t="s">
-        <v>1134</v>
+        <v>1138</v>
       </c>
       <c r="H288" s="1" t="s">
         <v>23</v>
@@ -16742,25 +16826,25 @@
     </row>
     <row r="289" spans="1:23">
       <c r="A289" t="s">
-        <v>1135</v>
+        <v>1139</v>
       </c>
       <c r="B289" t="s">
-        <v>1136</v>
+        <v>1140</v>
       </c>
       <c r="C289" t="s">
-        <v>1137</v>
-      </c>
-      <c r="D289" t="s">
-        <v>47</v>
-      </c>
-      <c r="E289" t="s">
-        <v>47</v>
+        <v>1141</v>
+      </c>
+      <c r="D289">
+        <v>34</v>
+      </c>
+      <c r="E289">
+        <v>5</v>
       </c>
       <c r="F289">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="G289" t="s">
-        <v>1138</v>
+        <v>1142</v>
       </c>
       <c r="H289" s="1" t="s">
         <v>23</v>
@@ -16771,25 +16855,25 @@
     </row>
     <row r="290" spans="1:23">
       <c r="A290" t="s">
-        <v>1139</v>
+        <v>602</v>
       </c>
       <c r="B290" t="s">
-        <v>1140</v>
+        <v>1143</v>
       </c>
       <c r="C290" t="s">
-        <v>1141</v>
+        <v>1144</v>
       </c>
       <c r="D290">
-        <v>34</v>
-      </c>
-      <c r="E290">
-        <v>5</v>
+        <v>579</v>
+      </c>
+      <c r="E290" t="s">
+        <v>47</v>
       </c>
       <c r="F290">
         <v>2024</v>
       </c>
       <c r="G290" t="s">
-        <v>1142</v>
+        <v>605</v>
       </c>
       <c r="H290" s="1" t="s">
         <v>23</v>
@@ -16800,25 +16884,25 @@
     </row>
     <row r="291" spans="1:23">
       <c r="A291" t="s">
-        <v>602</v>
+        <v>1145</v>
       </c>
       <c r="B291" t="s">
-        <v>1143</v>
+        <v>1146</v>
       </c>
       <c r="C291" t="s">
-        <v>1144</v>
+        <v>35</v>
       </c>
       <c r="D291">
-        <v>579</v>
-      </c>
-      <c r="E291" t="s">
-        <v>47</v>
+        <v>14</v>
+      </c>
+      <c r="E291">
+        <v>8</v>
       </c>
       <c r="F291">
         <v>2024</v>
       </c>
       <c r="G291" t="s">
-        <v>605</v>
+        <v>1147</v>
       </c>
       <c r="H291" s="1" t="s">
         <v>23</v>
@@ -16827,61 +16911,73 @@
         <v>668</v>
       </c>
     </row>
-    <row r="292" spans="1:23">
-      <c r="A292" t="s">
-        <v>1145</v>
-      </c>
-      <c r="B292" t="s">
-        <v>1146</v>
-      </c>
-      <c r="C292" t="s">
-        <v>35</v>
-      </c>
-      <c r="D292">
-        <v>14</v>
-      </c>
-      <c r="E292">
-        <v>8</v>
-      </c>
-      <c r="F292">
-        <v>2024</v>
-      </c>
-      <c r="G292" t="s">
-        <v>1147</v>
-      </c>
-      <c r="H292" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I292" s="1" t="s">
+    <row r="294" spans="1:23" ht="16">
+      <c r="A294" s="4" t="s">
+        <v>1148</v>
+      </c>
+    </row>
+    <row r="295" spans="1:23">
+      <c r="A295" t="s">
+        <v>1149</v>
+      </c>
+      <c r="B295" t="s">
+        <v>1150</v>
+      </c>
+      <c r="C295" t="s">
+        <v>93</v>
+      </c>
+      <c r="D295">
+        <v>12</v>
+      </c>
+      <c r="E295">
+        <v>1</v>
+      </c>
+      <c r="F295">
+        <v>2024</v>
+      </c>
+      <c r="G295" s="7" t="s">
+        <v>1151</v>
+      </c>
+      <c r="H295" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I295" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J295" s="1" t="s">
         <v>668</v>
       </c>
-    </row>
-    <row r="295" spans="1:23" ht="16">
-      <c r="A295" s="4" t="s">
-        <v>1148</v>
+      <c r="S295" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="V295" s="7" t="s">
+        <v>1152</v>
+      </c>
+      <c r="W295" s="7" t="s">
+        <v>304</v>
       </c>
     </row>
     <row r="296" spans="1:23">
       <c r="A296" t="s">
-        <v>1149</v>
+        <v>1153</v>
       </c>
       <c r="B296" t="s">
-        <v>1150</v>
+        <v>1154</v>
       </c>
       <c r="C296" t="s">
-        <v>93</v>
+        <v>1155</v>
       </c>
       <c r="D296">
-        <v>12</v>
-      </c>
-      <c r="E296">
-        <v>1</v>
+        <v>85</v>
+      </c>
+      <c r="E296" t="s">
+        <v>47</v>
       </c>
       <c r="F296">
-        <v>2024</v>
-      </c>
-      <c r="G296" s="7" t="s">
-        <v>1151</v>
+        <v>2025</v>
+      </c>
+      <c r="G296" t="s">
+        <v>578</v>
       </c>
       <c r="H296" s="1" t="s">
         <v>23</v>
@@ -16892,37 +16988,28 @@
       <c r="J296" s="1" t="s">
         <v>668</v>
       </c>
-      <c r="S296" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="V296" s="7" t="s">
-        <v>1152</v>
-      </c>
-      <c r="W296" s="7" t="s">
-        <v>304</v>
-      </c>
     </row>
     <row r="297" spans="1:23">
       <c r="A297" t="s">
-        <v>1153</v>
+        <v>1156</v>
       </c>
       <c r="B297" t="s">
-        <v>1154</v>
+        <v>1157</v>
       </c>
       <c r="C297" t="s">
-        <v>1155</v>
+        <v>1158</v>
       </c>
       <c r="D297">
-        <v>85</v>
-      </c>
-      <c r="E297" t="s">
-        <v>47</v>
+        <v>131</v>
+      </c>
+      <c r="E297">
+        <v>3</v>
       </c>
       <c r="F297">
         <v>2025</v>
       </c>
       <c r="G297" t="s">
-        <v>578</v>
+        <v>1159</v>
       </c>
       <c r="H297" s="1" t="s">
         <v>23</v>
@@ -16936,25 +17023,25 @@
     </row>
     <row r="298" spans="1:23">
       <c r="A298" t="s">
-        <v>1156</v>
+        <v>1160</v>
       </c>
       <c r="B298" t="s">
-        <v>1157</v>
+        <v>1161</v>
       </c>
       <c r="C298" t="s">
-        <v>1158</v>
-      </c>
-      <c r="D298">
-        <v>131</v>
-      </c>
-      <c r="E298">
-        <v>3</v>
+        <v>1162</v>
+      </c>
+      <c r="D298" t="s">
+        <v>47</v>
+      </c>
+      <c r="E298" t="s">
+        <v>47</v>
       </c>
       <c r="F298">
         <v>2025</v>
       </c>
       <c r="G298" t="s">
-        <v>1159</v>
+        <v>1163</v>
       </c>
       <c r="H298" s="1" t="s">
         <v>23</v>
@@ -16968,25 +17055,25 @@
     </row>
     <row r="299" spans="1:23">
       <c r="A299" t="s">
-        <v>1160</v>
+        <v>1164</v>
       </c>
       <c r="B299" t="s">
-        <v>1161</v>
+        <v>1165</v>
       </c>
       <c r="C299" t="s">
-        <v>1162</v>
-      </c>
-      <c r="D299" t="s">
-        <v>47</v>
-      </c>
-      <c r="E299" t="s">
-        <v>47</v>
+        <v>1166</v>
+      </c>
+      <c r="D299">
+        <v>49</v>
+      </c>
+      <c r="E299">
+        <v>8</v>
       </c>
       <c r="F299">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="G299" t="s">
-        <v>1163</v>
+        <v>526</v>
       </c>
       <c r="H299" s="1" t="s">
         <v>23</v>
@@ -17000,25 +17087,25 @@
     </row>
     <row r="300" spans="1:23">
       <c r="A300" t="s">
-        <v>1164</v>
+        <v>512</v>
       </c>
       <c r="B300" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="C300" t="s">
-        <v>1166</v>
+        <v>539</v>
       </c>
       <c r="D300">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="E300">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F300">
         <v>2024</v>
       </c>
       <c r="G300" t="s">
-        <v>526</v>
+        <v>1168</v>
       </c>
       <c r="H300" s="1" t="s">
         <v>23</v>
@@ -17032,25 +17119,25 @@
     </row>
     <row r="301" spans="1:23">
       <c r="A301" t="s">
-        <v>512</v>
+        <v>1169</v>
       </c>
       <c r="B301" t="s">
-        <v>1167</v>
+        <v>1170</v>
       </c>
       <c r="C301" t="s">
-        <v>539</v>
+        <v>1171</v>
       </c>
       <c r="D301">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E301">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F301">
         <v>2024</v>
       </c>
       <c r="G301" t="s">
-        <v>1168</v>
+        <v>1172</v>
       </c>
       <c r="H301" s="1" t="s">
         <v>23</v>
@@ -17064,16 +17151,16 @@
     </row>
     <row r="302" spans="1:23">
       <c r="A302" t="s">
-        <v>1169</v>
+        <v>565</v>
       </c>
       <c r="B302" t="s">
-        <v>1170</v>
+        <v>1173</v>
       </c>
       <c r="C302" t="s">
-        <v>1171</v>
+        <v>567</v>
       </c>
       <c r="D302">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="E302">
         <v>8</v>
@@ -17082,7 +17169,7 @@
         <v>2024</v>
       </c>
       <c r="G302" t="s">
-        <v>1172</v>
+        <v>1174</v>
       </c>
       <c r="H302" s="1" t="s">
         <v>23</v>
@@ -17096,25 +17183,25 @@
     </row>
     <row r="303" spans="1:23">
       <c r="A303" t="s">
-        <v>565</v>
+        <v>1175</v>
       </c>
       <c r="B303" t="s">
-        <v>1173</v>
+        <v>1176</v>
       </c>
       <c r="C303" t="s">
-        <v>567</v>
+        <v>1177</v>
       </c>
       <c r="D303">
-        <v>32</v>
-      </c>
-      <c r="E303">
-        <v>8</v>
+        <v>279</v>
+      </c>
+      <c r="E303" t="s">
+        <v>47</v>
       </c>
       <c r="F303">
         <v>2024</v>
       </c>
       <c r="G303" t="s">
-        <v>1174</v>
+        <v>1178</v>
       </c>
       <c r="H303" s="1" t="s">
         <v>23</v>
@@ -17128,25 +17215,25 @@
     </row>
     <row r="304" spans="1:23">
       <c r="A304" t="s">
-        <v>1175</v>
+        <v>1179</v>
       </c>
       <c r="B304" t="s">
-        <v>1176</v>
+        <v>1180</v>
       </c>
       <c r="C304" t="s">
-        <v>1177</v>
+        <v>380</v>
       </c>
       <c r="D304">
-        <v>279</v>
-      </c>
-      <c r="E304" t="s">
-        <v>47</v>
+        <v>379</v>
+      </c>
+      <c r="E304">
+        <v>1912</v>
       </c>
       <c r="F304">
         <v>2024</v>
       </c>
       <c r="G304" t="s">
-        <v>1178</v>
+        <v>545</v>
       </c>
       <c r="H304" s="1" t="s">
         <v>23</v>
@@ -17157,28 +17244,34 @@
       <c r="J304" s="1" t="s">
         <v>668</v>
       </c>
+      <c r="V304" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="W304" s="7" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="305" spans="1:23">
       <c r="A305" t="s">
-        <v>1179</v>
+        <v>1181</v>
       </c>
       <c r="B305" t="s">
-        <v>1180</v>
+        <v>1182</v>
       </c>
       <c r="C305" t="s">
-        <v>380</v>
-      </c>
-      <c r="D305">
-        <v>379</v>
-      </c>
-      <c r="E305">
-        <v>1912</v>
+        <v>1183</v>
+      </c>
+      <c r="D305" t="s">
+        <v>47</v>
+      </c>
+      <c r="E305" t="s">
+        <v>47</v>
       </c>
       <c r="F305">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="G305" t="s">
-        <v>545</v>
+        <v>1184</v>
       </c>
       <c r="H305" s="1" t="s">
         <v>23</v>
@@ -17189,34 +17282,28 @@
       <c r="J305" s="1" t="s">
         <v>668</v>
       </c>
-      <c r="V305" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="W305" s="7" t="s">
-        <v>82</v>
-      </c>
     </row>
     <row r="306" spans="1:23">
       <c r="A306" t="s">
-        <v>1181</v>
+        <v>1185</v>
       </c>
       <c r="B306" t="s">
-        <v>1182</v>
+        <v>1186</v>
       </c>
       <c r="C306" t="s">
-        <v>1183</v>
-      </c>
-      <c r="D306" t="s">
-        <v>47</v>
+        <v>1187</v>
+      </c>
+      <c r="D306">
+        <v>12</v>
       </c>
       <c r="E306" t="s">
         <v>47</v>
       </c>
       <c r="F306">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="G306" t="s">
-        <v>1184</v>
+        <v>1188</v>
       </c>
       <c r="H306" s="1" t="s">
         <v>23</v>
@@ -17230,25 +17317,25 @@
     </row>
     <row r="307" spans="1:23">
       <c r="A307" t="s">
-        <v>1185</v>
+        <v>558</v>
       </c>
       <c r="B307" t="s">
-        <v>1186</v>
+        <v>1189</v>
       </c>
       <c r="C307" t="s">
-        <v>1187</v>
+        <v>520</v>
       </c>
       <c r="D307">
         <v>12</v>
       </c>
-      <c r="E307" t="s">
-        <v>47</v>
+      <c r="E307">
+        <v>1</v>
       </c>
       <c r="F307">
         <v>2024</v>
       </c>
       <c r="G307" t="s">
-        <v>1188</v>
+        <v>560</v>
       </c>
       <c r="H307" s="1" t="s">
         <v>23</v>
@@ -17262,25 +17349,25 @@
     </row>
     <row r="308" spans="1:23">
       <c r="A308" t="s">
-        <v>558</v>
+        <v>1190</v>
       </c>
       <c r="B308" t="s">
-        <v>1189</v>
+        <v>1191</v>
       </c>
       <c r="C308" t="s">
-        <v>520</v>
+        <v>1192</v>
       </c>
       <c r="D308">
-        <v>12</v>
-      </c>
-      <c r="E308">
-        <v>1</v>
+        <v>82</v>
+      </c>
+      <c r="E308" t="s">
+        <v>47</v>
       </c>
       <c r="F308">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="G308" t="s">
-        <v>560</v>
+        <v>1193</v>
       </c>
       <c r="H308" s="1" t="s">
         <v>23</v>
@@ -17294,16 +17381,16 @@
     </row>
     <row r="309" spans="1:23">
       <c r="A309" t="s">
-        <v>1190</v>
+        <v>1194</v>
       </c>
       <c r="B309" t="s">
-        <v>1191</v>
+        <v>1195</v>
       </c>
       <c r="C309" t="s">
-        <v>1192</v>
+        <v>46</v>
       </c>
       <c r="D309">
-        <v>82</v>
+        <v>969</v>
       </c>
       <c r="E309" t="s">
         <v>47</v>
@@ -17312,7 +17399,7 @@
         <v>2025</v>
       </c>
       <c r="G309" t="s">
-        <v>1193</v>
+        <v>1196</v>
       </c>
       <c r="H309" s="1" t="s">
         <v>23</v>
@@ -17326,25 +17413,25 @@
     </row>
     <row r="310" spans="1:23">
       <c r="A310" t="s">
-        <v>1194</v>
+        <v>1197</v>
       </c>
       <c r="B310" t="s">
-        <v>1195</v>
+        <v>1198</v>
       </c>
       <c r="C310" t="s">
-        <v>46</v>
+        <v>539</v>
       </c>
       <c r="D310">
-        <v>969</v>
-      </c>
-      <c r="E310" t="s">
-        <v>47</v>
+        <v>12</v>
+      </c>
+      <c r="E310">
+        <v>1</v>
       </c>
       <c r="F310">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="G310" t="s">
-        <v>1196</v>
+        <v>1199</v>
       </c>
       <c r="H310" s="1" t="s">
         <v>23</v>
@@ -17355,28 +17442,34 @@
       <c r="J310" s="1" t="s">
         <v>668</v>
       </c>
+      <c r="V310" s="7" t="s">
+        <v>1200</v>
+      </c>
+      <c r="W310" s="7" t="s">
+        <v>1201</v>
+      </c>
     </row>
     <row r="311" spans="1:23">
       <c r="A311" t="s">
-        <v>1197</v>
+        <v>1202</v>
       </c>
       <c r="B311" t="s">
-        <v>1198</v>
+        <v>1203</v>
       </c>
       <c r="C311" t="s">
-        <v>539</v>
+        <v>1204</v>
       </c>
       <c r="D311">
-        <v>12</v>
+        <v>166</v>
       </c>
       <c r="E311">
         <v>1</v>
       </c>
       <c r="F311">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="G311" t="s">
-        <v>1199</v>
+        <v>1205</v>
       </c>
       <c r="H311" s="1" t="s">
         <v>23</v>
@@ -17388,33 +17481,33 @@
         <v>668</v>
       </c>
       <c r="V311" s="7" t="s">
-        <v>1200</v>
+        <v>1206</v>
       </c>
       <c r="W311" s="7" t="s">
-        <v>1201</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="312" spans="1:23">
       <c r="A312" t="s">
-        <v>1202</v>
+        <v>1208</v>
       </c>
       <c r="B312" t="s">
-        <v>1203</v>
+        <v>1209</v>
       </c>
       <c r="C312" t="s">
-        <v>1204</v>
+        <v>101</v>
       </c>
       <c r="D312">
-        <v>166</v>
+        <v>63</v>
       </c>
       <c r="E312">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F312">
         <v>2025</v>
       </c>
       <c r="G312" t="s">
-        <v>1205</v>
+        <v>1210</v>
       </c>
       <c r="H312" s="1" t="s">
         <v>23</v>
@@ -17425,34 +17518,28 @@
       <c r="J312" s="1" t="s">
         <v>668</v>
       </c>
-      <c r="V312" s="7" t="s">
-        <v>1206</v>
-      </c>
-      <c r="W312" s="7" t="s">
-        <v>1207</v>
-      </c>
     </row>
     <row r="313" spans="1:23">
       <c r="A313" t="s">
-        <v>1208</v>
+        <v>1211</v>
       </c>
       <c r="B313" t="s">
-        <v>1209</v>
+        <v>1212</v>
       </c>
       <c r="C313" t="s">
-        <v>101</v>
+        <v>238</v>
       </c>
       <c r="D313">
-        <v>63</v>
+        <v>15</v>
       </c>
       <c r="E313">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="F313">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="G313" t="s">
-        <v>1210</v>
+        <v>531</v>
       </c>
       <c r="H313" s="1" t="s">
         <v>23</v>
@@ -17463,28 +17550,34 @@
       <c r="J313" s="1" t="s">
         <v>668</v>
       </c>
+      <c r="V313" s="7" t="s">
+        <v>1213</v>
+      </c>
+      <c r="W313" s="7" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="314" spans="1:23">
       <c r="A314" t="s">
-        <v>1211</v>
+        <v>1214</v>
       </c>
       <c r="B314" t="s">
-        <v>1212</v>
+        <v>1215</v>
       </c>
       <c r="C314" t="s">
-        <v>238</v>
+        <v>1216</v>
       </c>
       <c r="D314">
-        <v>15</v>
+        <v>81</v>
       </c>
       <c r="E314">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F314">
         <v>2024</v>
       </c>
       <c r="G314" t="s">
-        <v>531</v>
+        <v>1217</v>
       </c>
       <c r="H314" s="1" t="s">
         <v>23</v>
@@ -17495,34 +17588,28 @@
       <c r="J314" s="1" t="s">
         <v>668</v>
       </c>
-      <c r="V314" s="7" t="s">
-        <v>1213</v>
-      </c>
-      <c r="W314" s="7" t="s">
-        <v>113</v>
-      </c>
     </row>
     <row r="315" spans="1:23">
       <c r="A315" t="s">
-        <v>1214</v>
+        <v>1218</v>
       </c>
       <c r="B315" t="s">
-        <v>1215</v>
+        <v>1219</v>
       </c>
       <c r="C315" t="s">
-        <v>1216</v>
+        <v>253</v>
       </c>
       <c r="D315">
-        <v>81</v>
-      </c>
-      <c r="E315">
-        <v>11</v>
+        <v>951</v>
+      </c>
+      <c r="E315" t="s">
+        <v>47</v>
       </c>
       <c r="F315">
         <v>2024</v>
       </c>
       <c r="G315" t="s">
-        <v>1217</v>
+        <v>1220</v>
       </c>
       <c r="H315" s="1" t="s">
         <v>23</v>
@@ -17536,25 +17623,25 @@
     </row>
     <row r="316" spans="1:23">
       <c r="A316" t="s">
-        <v>1218</v>
+        <v>537</v>
       </c>
       <c r="B316" t="s">
-        <v>1219</v>
+        <v>1221</v>
       </c>
       <c r="C316" t="s">
-        <v>253</v>
+        <v>514</v>
       </c>
       <c r="D316">
-        <v>951</v>
-      </c>
-      <c r="E316" t="s">
-        <v>47</v>
+        <v>12</v>
+      </c>
+      <c r="E316">
+        <v>1</v>
       </c>
       <c r="F316">
         <v>2024</v>
       </c>
       <c r="G316" t="s">
-        <v>1220</v>
+        <v>540</v>
       </c>
       <c r="H316" s="1" t="s">
         <v>23</v>
@@ -17568,25 +17655,25 @@
     </row>
     <row r="317" spans="1:23">
       <c r="A317" t="s">
-        <v>537</v>
+        <v>569</v>
       </c>
       <c r="B317" t="s">
-        <v>1221</v>
+        <v>1222</v>
       </c>
       <c r="C317" t="s">
-        <v>514</v>
+        <v>1057</v>
       </c>
       <c r="D317">
-        <v>12</v>
+        <v>70</v>
       </c>
       <c r="E317">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F317">
         <v>2024</v>
       </c>
       <c r="G317" t="s">
-        <v>540</v>
+        <v>571</v>
       </c>
       <c r="H317" s="1" t="s">
         <v>23</v>
@@ -17600,25 +17687,25 @@
     </row>
     <row r="318" spans="1:23">
       <c r="A318" t="s">
-        <v>569</v>
+        <v>1223</v>
       </c>
       <c r="B318" t="s">
-        <v>1222</v>
+        <v>1224</v>
       </c>
       <c r="C318" t="s">
-        <v>1057</v>
+        <v>1225</v>
       </c>
       <c r="D318">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="E318">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="F318">
         <v>2024</v>
       </c>
       <c r="G318" t="s">
-        <v>571</v>
+        <v>1226</v>
       </c>
       <c r="H318" s="1" t="s">
         <v>23</v>
@@ -17632,25 +17719,25 @@
     </row>
     <row r="319" spans="1:23">
       <c r="A319" t="s">
-        <v>1223</v>
+        <v>597</v>
       </c>
       <c r="B319" t="s">
-        <v>1224</v>
+        <v>1227</v>
       </c>
       <c r="C319" t="s">
-        <v>1225</v>
+        <v>551</v>
       </c>
       <c r="D319">
         <v>15</v>
       </c>
       <c r="E319">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="F319">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="G319" t="s">
-        <v>1226</v>
+        <v>599</v>
       </c>
       <c r="H319" s="1" t="s">
         <v>23</v>
@@ -17664,25 +17751,25 @@
     </row>
     <row r="320" spans="1:23">
       <c r="A320" t="s">
-        <v>597</v>
+        <v>1228</v>
       </c>
       <c r="B320" t="s">
-        <v>1227</v>
+        <v>1229</v>
       </c>
       <c r="C320" t="s">
-        <v>551</v>
+        <v>477</v>
       </c>
       <c r="D320">
-        <v>15</v>
+        <v>93</v>
       </c>
       <c r="E320">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F320">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="G320" t="s">
-        <v>599</v>
+        <v>1230</v>
       </c>
       <c r="H320" s="1" t="s">
         <v>23</v>
@@ -17694,27 +17781,27 @@
         <v>668</v>
       </c>
     </row>
-    <row r="321" spans="1:23">
-      <c r="A321" t="s">
-        <v>1228</v>
-      </c>
-      <c r="B321" t="s">
-        <v>1229</v>
-      </c>
-      <c r="C321" t="s">
-        <v>477</v>
-      </c>
-      <c r="D321">
+    <row r="321" spans="1:23" ht="15">
+      <c r="A321" s="16" t="s">
+        <v>1231</v>
+      </c>
+      <c r="B321" s="16" t="s">
+        <v>1232</v>
+      </c>
+      <c r="C321" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="E321">
-        <v>7</v>
-      </c>
-      <c r="F321">
-        <v>2024</v>
-      </c>
-      <c r="G321" t="s">
-        <v>1230</v>
+      <c r="D321" s="16">
+        <v>13</v>
+      </c>
+      <c r="E321" s="16">
+        <v>1</v>
+      </c>
+      <c r="F321" s="16">
+        <v>2025</v>
+      </c>
+      <c r="G321" s="16" t="s">
+        <v>1233</v>
       </c>
       <c r="H321" s="1" t="s">
         <v>23</v>
@@ -17726,103 +17813,103 @@
         <v>668</v>
       </c>
     </row>
-    <row r="322" spans="1:23" ht="15">
-      <c r="A322" s="16" t="s">
-        <v>1231</v>
-      </c>
-      <c r="B322" s="16" t="s">
-        <v>1232</v>
-      </c>
-      <c r="C322" s="16" t="s">
+    <row r="322" spans="1:23">
+      <c r="A322" t="s">
+        <v>1234</v>
+      </c>
+      <c r="B322" t="s">
+        <v>1235</v>
+      </c>
+      <c r="C322" t="s">
         <v>93</v>
       </c>
-      <c r="D322" s="16">
-        <v>13</v>
-      </c>
-      <c r="E322" s="16">
+      <c r="D322">
+        <v>12</v>
+      </c>
+      <c r="E322">
         <v>1</v>
       </c>
-      <c r="F322" s="16">
-        <v>2025</v>
-      </c>
-      <c r="G322" s="16" t="s">
-        <v>1233</v>
-      </c>
-      <c r="H322" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I322" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="J322" s="1" t="s">
+      <c r="F322">
+        <v>2024</v>
+      </c>
+      <c r="G322" t="s">
+        <v>1236</v>
+      </c>
+      <c r="H322" t="s">
+        <v>23</v>
+      </c>
+      <c r="I322" t="s">
+        <v>23</v>
+      </c>
+      <c r="J322" t="s">
         <v>668</v>
+      </c>
+      <c r="M322" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="T322" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="V322" s="7" t="s">
+        <v>1237</v>
+      </c>
+      <c r="W322" s="7" t="s">
+        <v>1238</v>
       </c>
     </row>
     <row r="323" spans="1:23">
       <c r="A323" t="s">
-        <v>1234</v>
+        <v>1239</v>
       </c>
       <c r="B323" t="s">
-        <v>1235</v>
+        <v>1240</v>
       </c>
       <c r="C323" t="s">
-        <v>93</v>
+        <v>775</v>
       </c>
       <c r="D323">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E323">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="F323">
         <v>2024</v>
       </c>
       <c r="G323" t="s">
-        <v>1236</v>
-      </c>
-      <c r="H323" t="s">
-        <v>23</v>
-      </c>
-      <c r="I323" t="s">
-        <v>23</v>
-      </c>
-      <c r="J323" t="s">
+        <v>1241</v>
+      </c>
+      <c r="H323" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I323" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J323" s="1" t="s">
         <v>668</v>
-      </c>
-      <c r="M323" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="T323" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="V323" s="7" t="s">
-        <v>1237</v>
-      </c>
-      <c r="W323" s="7" t="s">
-        <v>1238</v>
       </c>
     </row>
     <row r="324" spans="1:23">
       <c r="A324" t="s">
-        <v>1239</v>
+        <v>1242</v>
       </c>
       <c r="B324" t="s">
-        <v>1240</v>
+        <v>1243</v>
       </c>
       <c r="C324" t="s">
-        <v>775</v>
+        <v>230</v>
       </c>
       <c r="D324">
-        <v>16</v>
-      </c>
-      <c r="E324">
-        <v>23</v>
+        <v>302</v>
+      </c>
+      <c r="E324" t="s">
+        <v>47</v>
       </c>
       <c r="F324">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="G324" t="s">
-        <v>1241</v>
+        <v>1244</v>
       </c>
       <c r="H324" s="1" t="s">
         <v>23</v>
@@ -17836,25 +17923,25 @@
     </row>
     <row r="325" spans="1:23">
       <c r="A325" t="s">
-        <v>1242</v>
+        <v>572</v>
       </c>
       <c r="B325" t="s">
-        <v>1243</v>
+        <v>1245</v>
       </c>
       <c r="C325" t="s">
-        <v>230</v>
+        <v>551</v>
       </c>
       <c r="D325">
-        <v>302</v>
-      </c>
-      <c r="E325" t="s">
-        <v>47</v>
+        <v>15</v>
+      </c>
+      <c r="E325">
+        <v>1</v>
       </c>
       <c r="F325">
         <v>2025</v>
       </c>
       <c r="G325" t="s">
-        <v>1244</v>
+        <v>574</v>
       </c>
       <c r="H325" s="1" t="s">
         <v>23</v>
@@ -17868,13 +17955,13 @@
     </row>
     <row r="326" spans="1:23">
       <c r="A326" t="s">
-        <v>572</v>
+        <v>1246</v>
       </c>
       <c r="B326" t="s">
-        <v>1245</v>
+        <v>1247</v>
       </c>
       <c r="C326" t="s">
-        <v>551</v>
+        <v>35</v>
       </c>
       <c r="D326">
         <v>15</v>
@@ -17886,7 +17973,7 @@
         <v>2025</v>
       </c>
       <c r="G326" t="s">
-        <v>574</v>
+        <v>1248</v>
       </c>
       <c r="H326" s="1" t="s">
         <v>23</v>
@@ -17900,25 +17987,25 @@
     </row>
     <row r="327" spans="1:23">
       <c r="A327" t="s">
-        <v>1246</v>
+        <v>1249</v>
       </c>
       <c r="B327" t="s">
-        <v>1247</v>
+        <v>1250</v>
       </c>
       <c r="C327" t="s">
-        <v>35</v>
+        <v>230</v>
       </c>
       <c r="D327">
-        <v>15</v>
-      </c>
-      <c r="E327">
-        <v>1</v>
+        <v>302</v>
+      </c>
+      <c r="E327" t="s">
+        <v>47</v>
       </c>
       <c r="F327">
         <v>2025</v>
       </c>
       <c r="G327" t="s">
-        <v>1248</v>
+        <v>1251</v>
       </c>
       <c r="H327" s="1" t="s">
         <v>23</v>
@@ -17929,19 +18016,25 @@
       <c r="J327" s="1" t="s">
         <v>668</v>
       </c>
+      <c r="V327" s="7" t="s">
+        <v>1252</v>
+      </c>
+      <c r="W327" s="7" t="s">
+        <v>1253</v>
+      </c>
     </row>
     <row r="328" spans="1:23">
       <c r="A328" t="s">
-        <v>1249</v>
+        <v>1254</v>
       </c>
       <c r="B328" t="s">
-        <v>1250</v>
+        <v>1255</v>
       </c>
       <c r="C328" t="s">
-        <v>230</v>
-      </c>
-      <c r="D328">
-        <v>302</v>
+        <v>1204</v>
+      </c>
+      <c r="D328" t="s">
+        <v>47</v>
       </c>
       <c r="E328" t="s">
         <v>47</v>
@@ -17950,7 +18043,7 @@
         <v>2025</v>
       </c>
       <c r="G328" t="s">
-        <v>1251</v>
+        <v>1256</v>
       </c>
       <c r="H328" s="1" t="s">
         <v>23</v>
@@ -17962,33 +18055,33 @@
         <v>668</v>
       </c>
       <c r="V328" s="7" t="s">
-        <v>1252</v>
+        <v>1257</v>
       </c>
       <c r="W328" s="7" t="s">
-        <v>1253</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="329" spans="1:23">
       <c r="A329" t="s">
-        <v>1254</v>
+        <v>464</v>
       </c>
       <c r="B329" t="s">
-        <v>1255</v>
+        <v>465</v>
       </c>
       <c r="C329" t="s">
-        <v>1204</v>
-      </c>
-      <c r="D329" t="s">
-        <v>47</v>
-      </c>
-      <c r="E329" t="s">
-        <v>47</v>
+        <v>466</v>
+      </c>
+      <c r="D329">
+        <v>70</v>
+      </c>
+      <c r="E329">
+        <v>4</v>
       </c>
       <c r="F329">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="G329" t="s">
-        <v>1256</v>
+        <v>467</v>
       </c>
       <c r="H329" s="1" t="s">
         <v>23</v>
@@ -18000,33 +18093,33 @@
         <v>668</v>
       </c>
       <c r="V329" s="7" t="s">
-        <v>1257</v>
+        <v>1290</v>
       </c>
       <c r="W329" s="7" t="s">
-        <v>1258</v>
+        <v>1291</v>
       </c>
     </row>
     <row r="330" spans="1:23">
       <c r="A330" t="s">
-        <v>464</v>
+        <v>468</v>
       </c>
       <c r="B330" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
       <c r="C330" t="s">
-        <v>466</v>
+        <v>93</v>
       </c>
       <c r="D330">
-        <v>70</v>
+        <v>12</v>
       </c>
       <c r="E330">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F330">
         <v>2024</v>
       </c>
       <c r="G330" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="H330" s="1" t="s">
         <v>23</v>
@@ -18037,34 +18130,28 @@
       <c r="J330" s="1" t="s">
         <v>668</v>
       </c>
-      <c r="V330" s="7" t="s">
-        <v>1290</v>
-      </c>
-      <c r="W330" s="7" t="s">
-        <v>1291</v>
-      </c>
     </row>
     <row r="331" spans="1:23">
       <c r="A331" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="B331" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="C331" t="s">
-        <v>93</v>
+        <v>473</v>
       </c>
       <c r="D331">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E331">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F331">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="G331" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
       <c r="H331" s="1" t="s">
         <v>23</v>
@@ -18075,28 +18162,34 @@
       <c r="J331" s="1" t="s">
         <v>668</v>
       </c>
+      <c r="V331" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="W331" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="332" spans="1:23">
       <c r="A332" t="s">
-        <v>471</v>
+        <v>479</v>
       </c>
       <c r="B332" t="s">
-        <v>472</v>
+        <v>480</v>
       </c>
       <c r="C332" t="s">
-        <v>473</v>
+        <v>466</v>
       </c>
       <c r="D332">
-        <v>15</v>
+        <v>71</v>
       </c>
       <c r="E332">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F332">
         <v>2025</v>
       </c>
       <c r="G332" t="s">
-        <v>474</v>
+        <v>481</v>
       </c>
       <c r="H332" s="1" t="s">
         <v>23</v>
@@ -18108,33 +18201,33 @@
         <v>668</v>
       </c>
       <c r="V332" s="7" t="s">
-        <v>158</v>
+        <v>1295</v>
       </c>
       <c r="W332" s="7" t="s">
-        <v>159</v>
+        <v>1296</v>
       </c>
     </row>
     <row r="333" spans="1:23">
       <c r="A333" t="s">
-        <v>479</v>
+        <v>502</v>
       </c>
       <c r="B333" t="s">
-        <v>480</v>
+        <v>503</v>
       </c>
       <c r="C333" t="s">
-        <v>466</v>
+        <v>504</v>
       </c>
       <c r="D333">
-        <v>71</v>
-      </c>
-      <c r="E333">
-        <v>1</v>
+        <v>16</v>
+      </c>
+      <c r="E333" t="s">
+        <v>47</v>
       </c>
       <c r="F333">
         <v>2025</v>
       </c>
       <c r="G333" t="s">
-        <v>481</v>
+        <v>505</v>
       </c>
       <c r="H333" s="1" t="s">
         <v>23</v>
@@ -18145,48 +18238,10 @@
       <c r="J333" s="1" t="s">
         <v>668</v>
       </c>
-      <c r="V333" s="7" t="s">
-        <v>1295</v>
-      </c>
-      <c r="W333" s="7" t="s">
-        <v>1296</v>
-      </c>
-    </row>
-    <row r="334" spans="1:23">
-      <c r="A334" t="s">
-        <v>502</v>
-      </c>
-      <c r="B334" t="s">
-        <v>503</v>
-      </c>
-      <c r="C334" t="s">
-        <v>504</v>
-      </c>
-      <c r="D334">
-        <v>16</v>
-      </c>
-      <c r="E334" t="s">
-        <v>47</v>
-      </c>
-      <c r="F334">
-        <v>2025</v>
-      </c>
-      <c r="G334" t="s">
-        <v>505</v>
-      </c>
-      <c r="H334" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I334" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="J334" s="1" t="s">
-        <v>668</v>
-      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R2:R3 R297:R321 R324:R334 R5:R72" xr:uid="{AFB3D53A-87F1-495A-A1B6-17401F8CE4E8}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R2:R3 R296:R320 R323:R333 R5:R72" xr:uid="{AFB3D53A-87F1-495A-A1B6-17401F8CE4E8}"/>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -18198,43 +18253,43 @@
           <x14:formula1>
             <xm:f>'Keywords to use'!$C$10:$G$10</xm:f>
           </x14:formula1>
-          <xm:sqref>S296:S321 S324:S334 S2:S72</xm:sqref>
+          <xm:sqref>S295:S320 S323:S333 S2:S72</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9685C645-9740-4C33-B6F7-24E06EC9F241}">
           <x14:formula1>
             <xm:f>'Keywords to use'!$C$2:$D$2</xm:f>
           </x14:formula1>
-          <xm:sqref>K296:K321 K324:K334 K2:K72</xm:sqref>
+          <xm:sqref>K295:K320 K323:K333 K2:K72</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{AE68AA0A-296F-4174-BE8C-89FCADD7A5B0}">
           <x14:formula1>
             <xm:f>'Keywords to use'!$C$3:$E$3</xm:f>
           </x14:formula1>
-          <xm:sqref>L5:L12 L296:L298 L2:L3</xm:sqref>
+          <xm:sqref>L5:L12 L295:L297 L2:L3</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{6BD8521D-49AF-4E63-87D5-90C7B076EAED}">
           <x14:formula1>
             <xm:f>'Keywords to use'!$C$5:$E$5</xm:f>
           </x14:formula1>
-          <xm:sqref>O296:O321 O324:O334 O2:O72</xm:sqref>
+          <xm:sqref>O295:O320 O323:O333 O2:O72</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3CEC3D3B-863D-4293-AAA4-9BAA4918638C}">
           <x14:formula1>
             <xm:f>'Keywords to use'!$C$11:$E$11</xm:f>
           </x14:formula1>
-          <xm:sqref>T296:T321 T324:T334 T2:T72</xm:sqref>
+          <xm:sqref>T295:T320 T323:T333 T2:T72</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{6C78F827-A659-49E3-BB12-0411166A7866}">
           <x14:formula1>
             <xm:f>'Keywords to use'!$C$8:$L$8</xm:f>
           </x14:formula1>
-          <xm:sqref>Q296:R296 Q297:Q321 Q324:Q334 Q2:Q72</xm:sqref>
+          <xm:sqref>Q295:R295 Q296:Q320 Q323:Q333 Q2:Q72</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{5F77C6D1-45C7-48CF-AED8-63F987125AC4}">
           <x14:formula1>
             <xm:f>'Keywords to use'!$C$3:$F$3</xm:f>
           </x14:formula1>
-          <xm:sqref>L4 L299:L321 L324:L334 L13:L72</xm:sqref>
+          <xm:sqref>L4 L298:L320 L323:L333 L13:L72</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>